<commit_message>
actualizar archivos excel de pruebas
</commit_message>
<xml_diff>
--- a/tests/pytest/excel/archivos_de_prueba/clases_carrera_vacía.xlsx
+++ b/tests/pytest/excel/archivos_de_prueba/clases_carrera_vacía.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -120,7 +120,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -130,17 +130,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEB1C38"/>
-        <bgColor rgb="FFEB2242"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEB2242"/>
-        <bgColor rgb="FFEB1C38"/>
+        <bgColor rgb="FF993366"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -179,6 +173,15 @@
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
+      <top style="thin"/>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
@@ -248,7 +251,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -323,7 +326,7 @@
       <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FFEB2242"/>
+      <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
@@ -378,13 +381,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>472320</xdr:colOff>
+      <xdr:colOff>471960</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>9000</xdr:rowOff>
+      <xdr:rowOff>8640</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -394,7 +397,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="4617720" cy="637560"/>
+          <a:ext cx="4617360" cy="637200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -590,8 +593,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N202"/>
-  <sheetFormatPr defaultColWidth="8.56640625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M202"/>
+  <sheetFormatPr defaultColWidth="8.56640625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="27.27"/>
@@ -622,7 +625,6 @@
       <c r="K1" s="6"/>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4"/>
@@ -690,13 +692,14 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
+      <c r="B4" s="12"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="F4" s="13"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
       <c r="G4" s="14"/>
       <c r="H4" s="14"/>
-      <c r="I4" s="13"/>
+      <c r="I4" s="12"/>
       <c r="J4" s="13"/>
       <c r="K4" s="13"/>
       <c r="L4" s="13"/>
@@ -706,29 +709,31 @@
       <c r="A5" s="12"/>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
-      <c r="D5" s="13"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="13"/>
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12"/>
       <c r="B6" s="15"/>
       <c r="C6" s="15"/>
-      <c r="D6" s="13"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
       <c r="F6" s="13"/>
       <c r="G6" s="14"/>
       <c r="H6" s="14"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12"/>
@@ -3674,7 +3679,7 @@
   <mergeCells count="6">
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="E1:F1"/>
-    <mergeCell ref="G1:N1"/>
+    <mergeCell ref="G1:M1"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="J2:M2"/>
@@ -3707,7 +3712,7 @@
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>